<commit_message>
gpt-5 update, plus additional matches.
</commit_message>
<xml_diff>
--- a/UJ_ratings/UJ_map.xlsx
+++ b/UJ_ratings/UJ_map.xlsx
@@ -122,9 +122,6 @@
     <t>Crawfurd et al. 2023</t>
   </si>
   <si>
-    <t>How Much Would Reducing Lead Exposure Improve Children’s Learning in the Developing World?</t>
-  </si>
-  <si>
     <t>Walker et al. 2023</t>
   </si>
   <si>
@@ -252,6 +249,9 @@
   </si>
   <si>
     <t>research</t>
+  </si>
+  <si>
+    <t>How Much Would Reducing Lead Exposure Improve Childrens Learning in the Developing World?</t>
   </si>
 </sst>
 </file>
@@ -580,10 +580,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" t="s">
         <v>74</v>
-      </c>
-      <c r="B1" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
@@ -709,97 +709,97 @@
         <v>31</v>
       </c>
       <c r="B19" t="s">
-        <v>32</v>
+        <v>75</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
+        <v>32</v>
+      </c>
+      <c r="B20" t="s">
         <v>33</v>
-      </c>
-      <c r="B20" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
+        <v>34</v>
+      </c>
+      <c r="B21" t="s">
         <v>35</v>
-      </c>
-      <c r="B21" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
+        <v>37</v>
+      </c>
+      <c r="B23" t="s">
         <v>38</v>
-      </c>
-      <c r="B23" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
+        <v>39</v>
+      </c>
+      <c r="B24" t="s">
         <v>40</v>
-      </c>
-      <c r="B24" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
+        <v>41</v>
+      </c>
+      <c r="B25" t="s">
         <v>42</v>
-      </c>
-      <c r="B25" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
+        <v>43</v>
+      </c>
+      <c r="B26" t="s">
         <v>44</v>
-      </c>
-      <c r="B26" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B27" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
+        <v>46</v>
+      </c>
+      <c r="B28" t="s">
         <v>47</v>
-      </c>
-      <c r="B28" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
+        <v>48</v>
+      </c>
+      <c r="B29" t="s">
         <v>49</v>
-      </c>
-      <c r="B29" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
+        <v>50</v>
+      </c>
+      <c r="B30" t="s">
         <v>51</v>
-      </c>
-      <c r="B30" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" t="s">
         <v>53</v>
-      </c>
-      <c r="B31" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
@@ -809,23 +809,23 @@
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
+        <v>54</v>
+      </c>
+      <c r="B33" t="s">
         <v>55</v>
-      </c>
-      <c r="B33" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" t="s">
         <v>57</v>
-      </c>
-      <c r="B34" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.3">
@@ -833,62 +833,62 @@
         <v>2</v>
       </c>
       <c r="B36" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
+        <v>60</v>
+      </c>
+      <c r="B37" t="s">
         <v>61</v>
-      </c>
-      <c r="B37" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B38" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
+        <v>63</v>
+      </c>
+      <c r="B39" t="s">
         <v>64</v>
-      </c>
-      <c r="B39" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
+        <v>65</v>
+      </c>
+      <c r="B40" t="s">
         <v>66</v>
-      </c>
-      <c r="B40" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
+        <v>67</v>
+      </c>
+      <c r="B41" t="s">
         <v>68</v>
-      </c>
-      <c r="B41" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
+        <v>69</v>
+      </c>
+      <c r="B42" t="s">
         <v>70</v>
-      </c>
-      <c r="B42" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.3">
       <c r="B43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.3">

</xml_diff>